<commit_message>
Added correct beam structure
</commit_message>
<xml_diff>
--- a/Input files/Locations/Location details.xlsx
+++ b/Input files/Locations/Location details.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\velthj\Documents\GitHub\Context-analysis-codes\Input files\Locations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\velthj\Documents\GitHub\Solution-methodology-codes\Input files\Locations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3F0773C-513C-43CE-94FD-CD9B05A4C7AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D6054AD-9323-4473-8855-9FE7525553E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{45DC54C0-7ACB-4B87-A979-AF93CB064041}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{45DC54C0-7ACB-4B87-A979-AF93CB064041}"/>
   </bookViews>
   <sheets>
     <sheet name="Full Location Dataset" sheetId="1" r:id="rId1"/>
@@ -48123,7 +48123,6 @@
       <c r="L1164" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1164" xr:uid="{914862C9-AF29-4592-9C2E-1BD512AA1EBE}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Improve layout metrics and greedy outputs
Add a local-search pass in layout generation to reduce beam relocations and record before/after relocation metrics. Generate empty-location summaries by slot size, add space-utilization metrics and ranking inputs to final selection, and rename greedy pipeline outputs with `_greedy` suffixes so baseline and greedy artifacts stay separate. Also update the location details workbook to match the new pipeline inputs.
</commit_message>
<xml_diff>
--- a/Input files/Locations/Location details.xlsx
+++ b/Input files/Locations/Location details.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\velthj\Documents\GitHub\Solution-methodology-codes\Input files\Locations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E2C1E02-61C4-4DF9-8A39-E29EF69D0CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6F6CDE9-3F84-4DBE-8180-AFB5602A6911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{45DC54C0-7ACB-4B87-A979-AF93CB064041}"/>
   </bookViews>
@@ -4498,7 +4498,7 @@
         <v>234</v>
       </c>
       <c r="H10">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="I10" t="str">
         <f t="shared" si="3"/>
@@ -53448,7 +53448,7 @@
         <v>1106</v>
       </c>
       <c r="B1154" t="str">
-        <f t="shared" ref="B1154:B1217" si="93">LEFT(A1154,1)</f>
+        <f t="shared" ref="B1154:B1164" si="93">LEFT(A1154,1)</f>
         <v>K</v>
       </c>
       <c r="C1154" s="1" t="str">

</xml_diff>